<commit_message>
docs(readme): 更新 Action Table 示例图片路径
将 Action Table 示例图片的路径从 docs/action_table.png 修改为 imgs/action_table.png，确保图片正确显示。
</commit_message>
<xml_diff>
--- a/Course Project/Log/almighty/action table.xlsx
+++ b/Course Project/Log/almighty/action table.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kcfle\Documents\Jiangsu Classes\300 LEVEL\2nd Semester\Technology of Compilers\Lab\Course Project\Log\almighty\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C315807-A658-417E-8AA4-A5A21821434A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="28680" yWindow="3300" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -166,8 +172,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -230,13 +236,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -274,7 +288,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -308,6 +322,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -342,9 +357,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -517,11 +533,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="3" width="14.85546875" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" customWidth="1"/>
+    <col min="13" max="13" width="15.42578125" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -562,7 +589,6 @@
         <v>12</v>
       </c>
       <c r="O1" s="1">
-        <f/>
         <v>0</v>
       </c>
       <c r="P1" s="1" t="s">
@@ -572,7 +598,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -595,7 +621,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -624,7 +650,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -647,7 +673,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -670,7 +696,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -699,7 +725,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -728,7 +754,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -757,7 +783,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -786,7 +812,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -815,7 +841,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -838,7 +864,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -867,7 +893,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -899,7 +925,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -922,7 +948,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -948,7 +974,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -971,7 +997,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1000,7 +1026,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:17">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -1011,7 +1037,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -1034,7 +1060,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1045,7 +1071,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -1068,7 +1094,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -1079,7 +1105,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -1102,7 +1128,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:17">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -1131,7 +1157,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -1154,7 +1180,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:17">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -1165,7 +1191,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:17">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -1176,7 +1202,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:17">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -1184,7 +1210,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:17">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -1213,7 +1239,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:17">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -1221,7 +1247,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:17">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -1229,7 +1255,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:17">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>30</v>
       </c>

</xml_diff>